<commit_message>
﻿Manual commit: 2026/04/09 17:53:19
</commit_message>
<xml_diff>
--- a/仕様書/プロト仕様書-プログラマ-.xlsx
+++ b/仕様書/プロト仕様書-プログラマ-.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\HAL_3\kamigame\MagnetRush\仕様書\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{872066DA-01A8-4432-955D-016CF3D73C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A3AFFA6-C864-4B37-9E29-4B117FEA8505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2069,7 +2069,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2259,20 +2259,6 @@
     <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -2299,6 +2285,23 @@
     </xf>
     <xf numFmtId="0" fontId="41" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2620,32 +2623,32 @@
       <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="76" t="s">
+      <c r="C1" s="85" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
-      <c r="I1" s="74"/>
-      <c r="J1" s="74"/>
-      <c r="K1" s="74"/>
-      <c r="L1" s="74"/>
-      <c r="M1" s="74"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="76" t="s">
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
+      <c r="K1" s="83"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
+      <c r="N1" s="82"/>
+      <c r="O1" s="85" t="s">
         <v>62</v>
       </c>
-      <c r="P1" s="74"/>
-      <c r="Q1" s="74"/>
-      <c r="R1" s="74"/>
-      <c r="S1" s="74"/>
-      <c r="T1" s="74"/>
-      <c r="U1" s="74"/>
-      <c r="V1" s="74"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="73"/>
+      <c r="P1" s="83"/>
+      <c r="Q1" s="83"/>
+      <c r="R1" s="83"/>
+      <c r="S1" s="83"/>
+      <c r="T1" s="83"/>
+      <c r="U1" s="83"/>
+      <c r="V1" s="83"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="82"/>
     </row>
     <row r="2" spans="1:24" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3"/>
@@ -3237,12 +3240,12 @@
       </c>
     </row>
     <row r="14" spans="1:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="78" t="s">
+      <c r="A14" s="87" t="s">
         <v>327</v>
       </c>
-      <c r="B14" s="79"/>
-      <c r="C14" s="79"/>
-      <c r="D14" s="80"/>
+      <c r="B14" s="88"/>
+      <c r="C14" s="88"/>
+      <c r="D14" s="89"/>
     </row>
     <row r="15" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="26" t="s">
@@ -3444,33 +3447,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="75"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="73"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="82"/>
       <c r="AF1" s="24"/>
     </row>
     <row r="2" spans="1:32" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -4154,33 +4157,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="75"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="73"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="82"/>
       <c r="AF1" s="24"/>
     </row>
     <row r="2" spans="1:32" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -5049,33 +5052,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="75"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="73"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="82"/>
       <c r="AF1" s="24"/>
     </row>
     <row r="2" spans="1:32" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -5883,33 +5886,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="75"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="73"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="82"/>
       <c r="AF1" s="24"/>
     </row>
     <row r="2" spans="1:32" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7142,33 +7145,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="75"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="73"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="82"/>
       <c r="AF1" s="24"/>
     </row>
     <row r="2" spans="1:32" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7289,7 +7292,7 @@
         <v>35</v>
       </c>
       <c r="G3" s="53"/>
-      <c r="H3" s="81" t="s">
+      <c r="H3" s="71" t="s">
         <v>382</v>
       </c>
       <c r="I3" s="49" t="s">
@@ -7341,7 +7344,7 @@
         <v>35</v>
       </c>
       <c r="G4" s="57"/>
-      <c r="H4" s="82" t="s">
+      <c r="H4" s="72" t="s">
         <v>382</v>
       </c>
       <c r="I4" s="67" t="s">
@@ -7393,7 +7396,7 @@
       <c r="G5" s="54" t="s">
         <v>239</v>
       </c>
-      <c r="H5" s="82" t="s">
+      <c r="H5" s="72" t="s">
         <v>382</v>
       </c>
       <c r="I5" s="67" t="s">
@@ -7447,10 +7450,10 @@
       <c r="G6" s="54" t="s">
         <v>242</v>
       </c>
-      <c r="H6" s="82" t="s">
+      <c r="H6" s="72" t="s">
         <v>382</v>
       </c>
-      <c r="I6" s="86" t="s">
+      <c r="I6" s="76" t="s">
         <v>384</v>
       </c>
       <c r="J6" s="59"/>
@@ -7499,10 +7502,10 @@
       <c r="G7" s="54" t="s">
         <v>245</v>
       </c>
-      <c r="H7" s="82" t="s">
+      <c r="H7" s="72" t="s">
         <v>382</v>
       </c>
-      <c r="I7" s="87" t="s">
+      <c r="I7" s="77" t="s">
         <v>389</v>
       </c>
       <c r="J7" s="60" t="s">
@@ -7538,7 +7541,7 @@
       <c r="B8" s="20" t="s">
         <v>232</v>
       </c>
-      <c r="C8" s="89" t="s">
+      <c r="C8" s="79" t="s">
         <v>385</v>
       </c>
       <c r="D8" s="36" t="s">
@@ -7553,10 +7556,10 @@
       <c r="G8" s="54" t="s">
         <v>247</v>
       </c>
-      <c r="H8" s="82" t="s">
+      <c r="H8" s="72" t="s">
         <v>382</v>
       </c>
-      <c r="I8" s="88" t="s">
+      <c r="I8" s="78" t="s">
         <v>383</v>
       </c>
       <c r="J8" s="59"/>
@@ -7605,11 +7608,11 @@
       <c r="G9" s="55" t="s">
         <v>251</v>
       </c>
-      <c r="H9" s="83" t="s">
+      <c r="H9" s="73" t="s">
         <v>382</v>
       </c>
-      <c r="I9" s="49" t="s">
-        <v>36</v>
+      <c r="I9" s="90" t="s">
+        <v>383</v>
       </c>
       <c r="J9" s="59"/>
       <c r="K9" s="2"/>
@@ -7657,11 +7660,11 @@
       <c r="G10" s="54" t="s">
         <v>253</v>
       </c>
-      <c r="H10" s="82" t="s">
+      <c r="H10" s="72" t="s">
         <v>382</v>
       </c>
-      <c r="I10" s="51" t="s">
-        <v>36</v>
+      <c r="I10" s="78" t="s">
+        <v>383</v>
       </c>
       <c r="J10" s="60" t="s">
         <v>165</v>
@@ -7711,11 +7714,11 @@
       <c r="G11" s="54" t="s">
         <v>198</v>
       </c>
-      <c r="H11" s="82" t="s">
+      <c r="H11" s="72" t="s">
         <v>382</v>
       </c>
-      <c r="I11" s="51" t="s">
-        <v>36</v>
+      <c r="I11" s="78" t="s">
+        <v>383</v>
       </c>
       <c r="J11" s="59"/>
       <c r="K11" s="2"/>
@@ -7761,11 +7764,11 @@
         <v>42</v>
       </c>
       <c r="G12" s="53"/>
-      <c r="H12" s="85" t="s">
+      <c r="H12" s="75" t="s">
         <v>382</v>
       </c>
-      <c r="I12" s="49" t="s">
-        <v>36</v>
+      <c r="I12" s="90" t="s">
+        <v>383</v>
       </c>
       <c r="J12" s="59"/>
       <c r="K12" s="2"/>
@@ -7813,7 +7816,7 @@
       <c r="G13" s="54" t="s">
         <v>261</v>
       </c>
-      <c r="H13" s="84" t="s">
+      <c r="H13" s="74" t="s">
         <v>382</v>
       </c>
       <c r="I13" s="51" t="s">
@@ -7867,11 +7870,11 @@
       <c r="G14" s="54" t="s">
         <v>264</v>
       </c>
-      <c r="H14" s="84" t="s">
+      <c r="H14" s="74" t="s">
         <v>382</v>
       </c>
-      <c r="I14" s="51" t="s">
-        <v>36</v>
+      <c r="I14" s="78" t="s">
+        <v>383</v>
       </c>
       <c r="J14" s="60" t="s">
         <v>165</v>
@@ -7921,11 +7924,11 @@
       <c r="G15" s="54" t="s">
         <v>267</v>
       </c>
-      <c r="H15" s="84" t="s">
+      <c r="H15" s="74" t="s">
         <v>382</v>
       </c>
-      <c r="I15" s="51" t="s">
-        <v>36</v>
+      <c r="I15" s="78" t="s">
+        <v>383</v>
       </c>
       <c r="J15" s="59"/>
       <c r="K15" s="2"/>
@@ -8017,33 +8020,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="75"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="73"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="82"/>
       <c r="AF1" s="24"/>
     </row>
     <row r="2" spans="1:32" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8386,33 +8389,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="75"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="73"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="82"/>
       <c r="AF1" s="24"/>
     </row>
     <row r="2" spans="1:32" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8874,33 +8877,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="75"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="73"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="83"/>
+      <c r="X1" s="83"/>
+      <c r="Y1" s="83"/>
+      <c r="Z1" s="83"/>
+      <c r="AA1" s="83"/>
+      <c r="AB1" s="83"/>
+      <c r="AC1" s="83"/>
+      <c r="AD1" s="83"/>
+      <c r="AE1" s="82"/>
       <c r="AF1" s="24"/>
     </row>
     <row r="2" spans="1:32" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
﻿Manual commit: 2026/04/09 21:54:50
</commit_message>
<xml_diff>
--- a/仕様書/プロト仕様書-プログラマ-.xlsx
+++ b/仕様書/プロト仕様書-プログラマ-.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\HAL_3\kamigame\MagnetRush\仕様書\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A3AFFA6-C864-4B37-9E29-4B117FEA8505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3581660-26E1-4E09-B939-8DAC507D0260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7819,8 +7819,8 @@
       <c r="H13" s="74" t="s">
         <v>382</v>
       </c>
-      <c r="I13" s="51" t="s">
-        <v>36</v>
+      <c r="I13" s="78" t="s">
+        <v>383</v>
       </c>
       <c r="J13" s="60" t="s">
         <v>44</v>

</xml_diff>